<commit_message>
feat: upgrade HSE dashboard to v3 — live formulas, Candara font, charts, protection
- Replaced static v2 with fully automated v3: all KPIs use SUMPRODUCT formulas
- Added 6 live charts on dashboard (monthly incidents, inspection scores, action/training/risk breakdowns)
- Switched font to Candara across all sheets
- Locked dashboard design (sheet protection) — charts/layout can't be accidentally moved
- Filter cells explicitly unlocked so Year/Month/Dept/Location dropdowns stay editable
- Fixed chart row heights (10pt × 20 rows matches 268px chart height)
- INCIDENTS, INSPECTIONS, TRAINING, ACTIONS, RISK REGISTER, ENVIRONMENT all have dropdowns + conditional formatting + auto-calculate formulas

https://claude.ai/code/session_01GWgEEwfYnssivXBBGdjyqm
</commit_message>
<xml_diff>
--- a/static/resources/HSE-Complete-Dashboard.xlsx
+++ b/static/resources/HSE-Complete-Dashboard.xlsx
@@ -884,7 +884,7 @@
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="33">
+  <fonts count="34">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -896,246 +896,221 @@
       <b/>
       <sz val="8"/>
       <color rgb="FF00FF87"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <color rgb="FFFF3333"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FFDDDDDD"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <color rgb="FF00FF87"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <color rgb="FF00D4C8"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <color rgb="FFFFD60A"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <color rgb="FFFF8C00"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="22"/>
       <color rgb="FF00FF87"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF6A8FAA"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF00FF87"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FF6A8FAA"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFD60A"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFD60A"/>
+      <name val="Candara"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="13"/>
       <color rgb="FFFF3333"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="20"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="13"/>
       <color rgb="FFFF8C00"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="13"/>
       <color rgb="FF00FF87"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="13"/>
       <color rgb="FF00D4C8"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="13"/>
       <color rgb="FF9B6DFF"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="13"/>
       <color rgb="FFFFD60A"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="8"/>
       <color rgb="FF6A8FAA"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
       <sz val="7"/>
       <color rgb="FFFF3333"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
       <sz val="7"/>
       <color rgb="FFFF8C00"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
       <sz val="7"/>
       <color rgb="FF00FF87"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
       <sz val="7"/>
       <color rgb="FF00D4C8"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
       <sz val="7"/>
       <color rgb="FF9B6DFF"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
       <sz val="7"/>
       <color rgb="FFFFD60A"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FF00FF87"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="8"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="7"/>
       <color rgb="FF6A8FAA"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <color rgb="FF00FF87"/>
-      <name val="Calibri"/>
+      <name val="Candara"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="13">
@@ -1254,7 +1229,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1316,10 +1291,11 @@
     <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1361,28 +1337,31 @@
     <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2815,8 +2794,8 @@
     <xdr:to>
       <xdr:col>16</xdr:col>
       <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2845,8 +2824,8 @@
     <xdr:to>
       <xdr:col>28</xdr:col>
       <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2875,8 +2854,8 @@
     <xdr:to>
       <xdr:col>40</xdr:col>
       <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2905,8 +2884,8 @@
     <xdr:to>
       <xdr:col>16</xdr:col>
       <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>76</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2935,8 +2914,8 @@
     <xdr:to>
       <xdr:col>28</xdr:col>
       <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>76</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2965,8 +2944,8 @@
     <xdr:to>
       <xdr:col>40</xdr:col>
       <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>76</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -22262,568 +22241,568 @@
       <c r="C7" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="21"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
       <c r="I7" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="J7" s="21"/>
-      <c r="K7" s="21"/>
-      <c r="L7" s="21"/>
-      <c r="M7" s="21"/>
-      <c r="N7" s="21"/>
-      <c r="O7" s="21"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="22"/>
+      <c r="L7" s="22"/>
+      <c r="M7" s="22"/>
+      <c r="N7" s="22"/>
+      <c r="O7" s="22"/>
       <c r="P7" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="21"/>
-      <c r="S7" s="21"/>
-      <c r="T7" s="21"/>
-      <c r="U7" s="21"/>
+      <c r="Q7" s="22"/>
+      <c r="R7" s="22"/>
+      <c r="S7" s="22"/>
+      <c r="T7" s="22"/>
+      <c r="U7" s="22"/>
       <c r="V7" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="W7" s="21"/>
-      <c r="X7" s="21"/>
-      <c r="Y7" s="21"/>
-      <c r="Z7" s="21"/>
-      <c r="AA7" s="21"/>
-      <c r="AB7" s="21"/>
+      <c r="W7" s="22"/>
+      <c r="X7" s="22"/>
+      <c r="Y7" s="22"/>
+      <c r="Z7" s="22"/>
+      <c r="AA7" s="22"/>
+      <c r="AB7" s="22"/>
     </row>
     <row r="8" spans="3:44" ht="4" customHeight="1"/>
     <row r="9" spans="3:44" ht="12" customHeight="1"/>
     <row r="10" spans="3:44" ht="18" customHeight="1"/>
     <row r="11" spans="3:44" ht="18" customHeight="1">
-      <c r="D11" s="22" t="s">
+      <c r="D11" s="23" t="s">
         <v>226</v>
       </c>
-      <c r="E11" s="22"/>
-      <c r="F11" s="23">
+      <c r="E11" s="23"/>
+      <c r="F11" s="24">
         <f>SUMPRODUCT((IncidentsTable[Date]&lt;&gt;"")*IF($C$7="All",1,(IncidentsTable[_Year]=IF(ISNUMBER($C$7),$C$7,VALUE($C$7))))*IF($I$7="All",1,(IncidentsTable[_Month]=$I$7))*IF($P$7="All",1,(IncidentsTable[Department]=$P$7))*IF($V$7="All",1,(IncidentsTable[Location]=$V$7)))</f>
         <v>0</v>
       </c>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
-      <c r="K11" s="24" t="s">
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="24"/>
+      <c r="K11" s="25" t="s">
         <v>229</v>
       </c>
-      <c r="L11" s="24"/>
-      <c r="M11" s="23">
+      <c r="L11" s="25"/>
+      <c r="M11" s="24">
         <f>SUMPRODUCT((IncidentsTable[Type]="Near Miss")*IF($C$7="All",1,(IncidentsTable[_Year]=IF(ISNUMBER($C$7),$C$7,VALUE($C$7))))*IF($I$7="All",1,(IncidentsTable[_Month]=$I$7))*IF($P$7="All",1,(IncidentsTable[Department]=$P$7))*IF($V$7="All",1,(IncidentsTable[Location]=$V$7)))</f>
         <v>0</v>
       </c>
-      <c r="N11" s="23"/>
-      <c r="O11" s="23"/>
-      <c r="P11" s="23"/>
-      <c r="R11" s="25" t="s">
+      <c r="N11" s="24"/>
+      <c r="O11" s="24"/>
+      <c r="P11" s="24"/>
+      <c r="R11" s="26" t="s">
         <v>230</v>
       </c>
-      <c r="S11" s="25"/>
-      <c r="T11" s="23">
+      <c r="S11" s="26"/>
+      <c r="T11" s="24">
         <f>IFERROR(SUMPRODUCT((InspectionsTable[Score %]&lt;&gt;"")*IF($C$7="All",1,(InspectionsTable[_Year]=IF(ISNUMBER($C$7),$C$7,VALUE($C$7))))*IF($I$7="All",1,(InspectionsTable[_Month]=$I$7))*IF($P$7="All",1,(InspectionsTable[Department]=$P$7))*(InspectionsTable[Score %]))/SUMPRODUCT((InspectionsTable[Score %]&lt;&gt;"")*IF($C$7="All",1,(InspectionsTable[_Year]=IF(ISNUMBER($C$7),$C$7,VALUE($C$7))))*IF($I$7="All",1,(InspectionsTable[_Month]=$I$7))*IF($P$7="All",1,(InspectionsTable[Department]=$P$7))),"--")</f>
         <v>0</v>
       </c>
-      <c r="U11" s="23"/>
-      <c r="V11" s="23"/>
-      <c r="W11" s="23"/>
-      <c r="Y11" s="26" t="s">
+      <c r="U11" s="24"/>
+      <c r="V11" s="24"/>
+      <c r="W11" s="24"/>
+      <c r="Y11" s="27" t="s">
         <v>232</v>
       </c>
-      <c r="Z11" s="26"/>
-      <c r="AA11" s="23">
+      <c r="Z11" s="27"/>
+      <c r="AA11" s="24">
         <f>IFERROR(SUMPRODUCT((TrainingTable[Auto-Status]="Complete")*IF($P$7="All",1,(TrainingTable[Department]=$P$7)))/SUMPRODUCT((TrainingTable[Auto-Status]&lt;&gt;"")*IF($P$7="All",1,(TrainingTable[Department]=$P$7)))*100,"--")</f>
         <v>0</v>
       </c>
-      <c r="AB11" s="23"/>
-      <c r="AC11" s="23"/>
-      <c r="AD11" s="23"/>
-      <c r="AF11" s="27" t="s">
+      <c r="AB11" s="24"/>
+      <c r="AC11" s="24"/>
+      <c r="AD11" s="24"/>
+      <c r="AF11" s="28" t="s">
         <v>234</v>
       </c>
-      <c r="AG11" s="27"/>
-      <c r="AH11" s="23">
+      <c r="AG11" s="28"/>
+      <c r="AH11" s="24">
         <f>IFERROR(SUMPRODUCT((InspectionsTable[Score %]&gt;=90)*IF($C$7="All",1,(InspectionsTable[_Year]=IF(ISNUMBER($C$7),$C$7,VALUE($C$7))))*IF($I$7="All",1,(InspectionsTable[_Month]=$I$7))*IF($P$7="All",1,(InspectionsTable[Department]=$P$7)))/SUMPRODUCT((InspectionsTable[Score %]&lt;&gt;"")*IF($C$7="All",1,(InspectionsTable[_Year]=IF(ISNUMBER($C$7),$C$7,VALUE($C$7))))*IF($I$7="All",1,(InspectionsTable[_Month]=$I$7))*IF($P$7="All",1,(InspectionsTable[Department]=$P$7)))*100,"--")</f>
         <v>0</v>
       </c>
-      <c r="AI11" s="23"/>
-      <c r="AJ11" s="23"/>
-      <c r="AK11" s="23"/>
-      <c r="AM11" s="28" t="s">
+      <c r="AI11" s="24"/>
+      <c r="AJ11" s="24"/>
+      <c r="AK11" s="24"/>
+      <c r="AM11" s="29" t="s">
         <v>236</v>
       </c>
-      <c r="AN11" s="28"/>
-      <c r="AO11" s="23">
+      <c r="AN11" s="29"/>
+      <c r="AO11" s="24">
         <f>SUMPRODUCT((ActionsTable[Status]&lt;&gt;"Done")*(ActionsTable[Status]&lt;&gt;"Closed")*(ActionsTable[Status]&lt;&gt;"")*IF($P$7="All",1,(ActionsTable[Department]=$P$7)))</f>
         <v>0</v>
       </c>
-      <c r="AP11" s="23"/>
-      <c r="AQ11" s="23"/>
-      <c r="AR11" s="23"/>
+      <c r="AP11" s="24"/>
+      <c r="AQ11" s="24"/>
+      <c r="AR11" s="24"/>
     </row>
     <row r="12" spans="3:44" ht="18" customHeight="1">
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="23"/>
-      <c r="I12" s="23"/>
-      <c r="K12" s="24"/>
-      <c r="L12" s="24"/>
-      <c r="M12" s="23"/>
-      <c r="N12" s="23"/>
-      <c r="O12" s="23"/>
-      <c r="P12" s="23"/>
-      <c r="R12" s="25"/>
-      <c r="S12" s="25"/>
-      <c r="T12" s="23"/>
-      <c r="U12" s="23"/>
-      <c r="V12" s="23"/>
-      <c r="W12" s="23"/>
-      <c r="Y12" s="26"/>
-      <c r="Z12" s="26"/>
-      <c r="AA12" s="23"/>
-      <c r="AB12" s="23"/>
-      <c r="AC12" s="23"/>
-      <c r="AD12" s="23"/>
-      <c r="AF12" s="27"/>
-      <c r="AG12" s="27"/>
-      <c r="AH12" s="23"/>
-      <c r="AI12" s="23"/>
-      <c r="AJ12" s="23"/>
-      <c r="AK12" s="23"/>
-      <c r="AM12" s="28"/>
-      <c r="AN12" s="28"/>
-      <c r="AO12" s="23"/>
-      <c r="AP12" s="23"/>
-      <c r="AQ12" s="23"/>
-      <c r="AR12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="24"/>
+      <c r="K12" s="25"/>
+      <c r="L12" s="25"/>
+      <c r="M12" s="24"/>
+      <c r="N12" s="24"/>
+      <c r="O12" s="24"/>
+      <c r="P12" s="24"/>
+      <c r="R12" s="26"/>
+      <c r="S12" s="26"/>
+      <c r="T12" s="24"/>
+      <c r="U12" s="24"/>
+      <c r="V12" s="24"/>
+      <c r="W12" s="24"/>
+      <c r="Y12" s="27"/>
+      <c r="Z12" s="27"/>
+      <c r="AA12" s="24"/>
+      <c r="AB12" s="24"/>
+      <c r="AC12" s="24"/>
+      <c r="AD12" s="24"/>
+      <c r="AF12" s="28"/>
+      <c r="AG12" s="28"/>
+      <c r="AH12" s="24"/>
+      <c r="AI12" s="24"/>
+      <c r="AJ12" s="24"/>
+      <c r="AK12" s="24"/>
+      <c r="AM12" s="29"/>
+      <c r="AN12" s="29"/>
+      <c r="AO12" s="24"/>
+      <c r="AP12" s="24"/>
+      <c r="AQ12" s="24"/>
+      <c r="AR12" s="24"/>
     </row>
     <row r="13" spans="3:44" ht="18" customHeight="1">
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="23"/>
-      <c r="I13" s="23"/>
-      <c r="K13" s="24"/>
-      <c r="L13" s="24"/>
-      <c r="M13" s="23"/>
-      <c r="N13" s="23"/>
-      <c r="O13" s="23"/>
-      <c r="P13" s="23"/>
-      <c r="R13" s="25"/>
-      <c r="S13" s="25"/>
-      <c r="T13" s="23"/>
-      <c r="U13" s="23"/>
-      <c r="V13" s="23"/>
-      <c r="W13" s="23"/>
-      <c r="Y13" s="26"/>
-      <c r="Z13" s="26"/>
-      <c r="AA13" s="23"/>
-      <c r="AB13" s="23"/>
-      <c r="AC13" s="23"/>
-      <c r="AD13" s="23"/>
-      <c r="AF13" s="27"/>
-      <c r="AG13" s="27"/>
-      <c r="AH13" s="23"/>
-      <c r="AI13" s="23"/>
-      <c r="AJ13" s="23"/>
-      <c r="AK13" s="23"/>
-      <c r="AM13" s="28"/>
-      <c r="AN13" s="28"/>
-      <c r="AO13" s="23"/>
-      <c r="AP13" s="23"/>
-      <c r="AQ13" s="23"/>
-      <c r="AR13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
+      <c r="I13" s="24"/>
+      <c r="K13" s="25"/>
+      <c r="L13" s="25"/>
+      <c r="M13" s="24"/>
+      <c r="N13" s="24"/>
+      <c r="O13" s="24"/>
+      <c r="P13" s="24"/>
+      <c r="R13" s="26"/>
+      <c r="S13" s="26"/>
+      <c r="T13" s="24"/>
+      <c r="U13" s="24"/>
+      <c r="V13" s="24"/>
+      <c r="W13" s="24"/>
+      <c r="Y13" s="27"/>
+      <c r="Z13" s="27"/>
+      <c r="AA13" s="24"/>
+      <c r="AB13" s="24"/>
+      <c r="AC13" s="24"/>
+      <c r="AD13" s="24"/>
+      <c r="AF13" s="28"/>
+      <c r="AG13" s="28"/>
+      <c r="AH13" s="24"/>
+      <c r="AI13" s="24"/>
+      <c r="AJ13" s="24"/>
+      <c r="AK13" s="24"/>
+      <c r="AM13" s="29"/>
+      <c r="AN13" s="29"/>
+      <c r="AO13" s="24"/>
+      <c r="AP13" s="24"/>
+      <c r="AQ13" s="24"/>
+      <c r="AR13" s="24"/>
     </row>
     <row r="14" spans="3:44" ht="18" customHeight="1">
-      <c r="D14" s="29" t="s">
+      <c r="D14" s="30" t="s">
         <v>227</v>
       </c>
-      <c r="E14" s="29"/>
-      <c r="F14" s="29"/>
-      <c r="G14" s="29"/>
-      <c r="H14" s="29"/>
-      <c r="I14" s="29"/>
-      <c r="K14" s="29" t="s">
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="30"/>
+      <c r="K14" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="L14" s="29"/>
-      <c r="M14" s="29"/>
-      <c r="N14" s="29"/>
-      <c r="O14" s="29"/>
-      <c r="P14" s="29"/>
-      <c r="R14" s="29" t="s">
+      <c r="L14" s="30"/>
+      <c r="M14" s="30"/>
+      <c r="N14" s="30"/>
+      <c r="O14" s="30"/>
+      <c r="P14" s="30"/>
+      <c r="R14" s="30" t="s">
         <v>231</v>
       </c>
-      <c r="S14" s="29"/>
-      <c r="T14" s="29"/>
-      <c r="U14" s="29"/>
-      <c r="V14" s="29"/>
-      <c r="W14" s="29"/>
-      <c r="Y14" s="29" t="s">
+      <c r="S14" s="30"/>
+      <c r="T14" s="30"/>
+      <c r="U14" s="30"/>
+      <c r="V14" s="30"/>
+      <c r="W14" s="30"/>
+      <c r="Y14" s="30" t="s">
         <v>233</v>
       </c>
-      <c r="Z14" s="29"/>
-      <c r="AA14" s="29"/>
-      <c r="AB14" s="29"/>
-      <c r="AC14" s="29"/>
-      <c r="AD14" s="29"/>
-      <c r="AF14" s="29" t="s">
+      <c r="Z14" s="30"/>
+      <c r="AA14" s="30"/>
+      <c r="AB14" s="30"/>
+      <c r="AC14" s="30"/>
+      <c r="AD14" s="30"/>
+      <c r="AF14" s="30" t="s">
         <v>235</v>
       </c>
-      <c r="AG14" s="29"/>
-      <c r="AH14" s="29"/>
-      <c r="AI14" s="29"/>
-      <c r="AJ14" s="29"/>
-      <c r="AK14" s="29"/>
-      <c r="AM14" s="29" t="s">
+      <c r="AG14" s="30"/>
+      <c r="AH14" s="30"/>
+      <c r="AI14" s="30"/>
+      <c r="AJ14" s="30"/>
+      <c r="AK14" s="30"/>
+      <c r="AM14" s="30" t="s">
         <v>237</v>
       </c>
-      <c r="AN14" s="29"/>
-      <c r="AO14" s="29"/>
-      <c r="AP14" s="29"/>
-      <c r="AQ14" s="29"/>
-      <c r="AR14" s="29"/>
+      <c r="AN14" s="30"/>
+      <c r="AO14" s="30"/>
+      <c r="AP14" s="30"/>
+      <c r="AQ14" s="30"/>
+      <c r="AR14" s="30"/>
     </row>
     <row r="15" spans="3:44" ht="18" customHeight="1">
-      <c r="D15" s="29"/>
-      <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
-      <c r="G15" s="29"/>
-      <c r="H15" s="29"/>
-      <c r="I15" s="29"/>
-      <c r="K15" s="29"/>
-      <c r="L15" s="29"/>
-      <c r="M15" s="29"/>
-      <c r="N15" s="29"/>
-      <c r="O15" s="29"/>
-      <c r="P15" s="29"/>
-      <c r="R15" s="29"/>
-      <c r="S15" s="29"/>
-      <c r="T15" s="29"/>
-      <c r="U15" s="29"/>
-      <c r="V15" s="29"/>
-      <c r="W15" s="29"/>
-      <c r="Y15" s="29"/>
-      <c r="Z15" s="29"/>
-      <c r="AA15" s="29"/>
-      <c r="AB15" s="29"/>
-      <c r="AC15" s="29"/>
-      <c r="AD15" s="29"/>
-      <c r="AF15" s="29"/>
-      <c r="AG15" s="29"/>
-      <c r="AH15" s="29"/>
-      <c r="AI15" s="29"/>
-      <c r="AJ15" s="29"/>
-      <c r="AK15" s="29"/>
-      <c r="AM15" s="29"/>
-      <c r="AN15" s="29"/>
-      <c r="AO15" s="29"/>
-      <c r="AP15" s="29"/>
-      <c r="AQ15" s="29"/>
-      <c r="AR15" s="29"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="30"/>
+      <c r="K15" s="30"/>
+      <c r="L15" s="30"/>
+      <c r="M15" s="30"/>
+      <c r="N15" s="30"/>
+      <c r="O15" s="30"/>
+      <c r="P15" s="30"/>
+      <c r="R15" s="30"/>
+      <c r="S15" s="30"/>
+      <c r="T15" s="30"/>
+      <c r="U15" s="30"/>
+      <c r="V15" s="30"/>
+      <c r="W15" s="30"/>
+      <c r="Y15" s="30"/>
+      <c r="Z15" s="30"/>
+      <c r="AA15" s="30"/>
+      <c r="AB15" s="30"/>
+      <c r="AC15" s="30"/>
+      <c r="AD15" s="30"/>
+      <c r="AF15" s="30"/>
+      <c r="AG15" s="30"/>
+      <c r="AH15" s="30"/>
+      <c r="AI15" s="30"/>
+      <c r="AJ15" s="30"/>
+      <c r="AK15" s="30"/>
+      <c r="AM15" s="30"/>
+      <c r="AN15" s="30"/>
+      <c r="AO15" s="30"/>
+      <c r="AP15" s="30"/>
+      <c r="AQ15" s="30"/>
+      <c r="AR15" s="30"/>
     </row>
     <row r="16" spans="3:44" ht="18" customHeight="1">
-      <c r="D16" s="30" t="s">
+      <c r="D16" s="31" t="s">
         <v>228</v>
       </c>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="30"/>
-      <c r="I16" s="30"/>
-      <c r="K16" s="31" t="s">
+      <c r="E16" s="31"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="31"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="31"/>
+      <c r="K16" s="32" t="s">
         <v>228</v>
       </c>
-      <c r="L16" s="31"/>
-      <c r="M16" s="31"/>
-      <c r="N16" s="31"/>
-      <c r="O16" s="31"/>
-      <c r="P16" s="31"/>
-      <c r="R16" s="32" t="s">
+      <c r="L16" s="32"/>
+      <c r="M16" s="32"/>
+      <c r="N16" s="32"/>
+      <c r="O16" s="32"/>
+      <c r="P16" s="32"/>
+      <c r="R16" s="33" t="s">
         <v>228</v>
       </c>
-      <c r="S16" s="32"/>
-      <c r="T16" s="32"/>
-      <c r="U16" s="32"/>
-      <c r="V16" s="32"/>
-      <c r="W16" s="32"/>
-      <c r="Y16" s="33" t="s">
+      <c r="S16" s="33"/>
+      <c r="T16" s="33"/>
+      <c r="U16" s="33"/>
+      <c r="V16" s="33"/>
+      <c r="W16" s="33"/>
+      <c r="Y16" s="34" t="s">
         <v>228</v>
       </c>
-      <c r="Z16" s="33"/>
-      <c r="AA16" s="33"/>
-      <c r="AB16" s="33"/>
-      <c r="AC16" s="33"/>
-      <c r="AD16" s="33"/>
-      <c r="AF16" s="34" t="s">
+      <c r="Z16" s="34"/>
+      <c r="AA16" s="34"/>
+      <c r="AB16" s="34"/>
+      <c r="AC16" s="34"/>
+      <c r="AD16" s="34"/>
+      <c r="AF16" s="35" t="s">
         <v>228</v>
       </c>
-      <c r="AG16" s="34"/>
-      <c r="AH16" s="34"/>
-      <c r="AI16" s="34"/>
-      <c r="AJ16" s="34"/>
-      <c r="AK16" s="34"/>
-      <c r="AM16" s="35" t="s">
+      <c r="AG16" s="35"/>
+      <c r="AH16" s="35"/>
+      <c r="AI16" s="35"/>
+      <c r="AJ16" s="35"/>
+      <c r="AK16" s="35"/>
+      <c r="AM16" s="36" t="s">
         <v>228</v>
       </c>
-      <c r="AN16" s="35"/>
-      <c r="AO16" s="35"/>
-      <c r="AP16" s="35"/>
-      <c r="AQ16" s="35"/>
-      <c r="AR16" s="35"/>
+      <c r="AN16" s="36"/>
+      <c r="AO16" s="36"/>
+      <c r="AP16" s="36"/>
+      <c r="AQ16" s="36"/>
+      <c r="AR16" s="36"/>
     </row>
     <row r="17" spans="3:44" ht="18" customHeight="1">
-      <c r="D17" s="30"/>
-      <c r="E17" s="30"/>
-      <c r="F17" s="30"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="30"/>
-      <c r="I17" s="30"/>
-      <c r="K17" s="31"/>
-      <c r="L17" s="31"/>
-      <c r="M17" s="31"/>
-      <c r="N17" s="31"/>
-      <c r="O17" s="31"/>
-      <c r="P17" s="31"/>
-      <c r="R17" s="32"/>
-      <c r="S17" s="32"/>
-      <c r="T17" s="32"/>
-      <c r="U17" s="32"/>
-      <c r="V17" s="32"/>
-      <c r="W17" s="32"/>
-      <c r="Y17" s="33"/>
-      <c r="Z17" s="33"/>
-      <c r="AA17" s="33"/>
-      <c r="AB17" s="33"/>
-      <c r="AC17" s="33"/>
-      <c r="AD17" s="33"/>
-      <c r="AF17" s="34"/>
-      <c r="AG17" s="34"/>
-      <c r="AH17" s="34"/>
-      <c r="AI17" s="34"/>
-      <c r="AJ17" s="34"/>
-      <c r="AK17" s="34"/>
-      <c r="AM17" s="35"/>
-      <c r="AN17" s="35"/>
-      <c r="AO17" s="35"/>
-      <c r="AP17" s="35"/>
-      <c r="AQ17" s="35"/>
-      <c r="AR17" s="35"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="31"/>
+      <c r="G17" s="31"/>
+      <c r="H17" s="31"/>
+      <c r="I17" s="31"/>
+      <c r="K17" s="32"/>
+      <c r="L17" s="32"/>
+      <c r="M17" s="32"/>
+      <c r="N17" s="32"/>
+      <c r="O17" s="32"/>
+      <c r="P17" s="32"/>
+      <c r="R17" s="33"/>
+      <c r="S17" s="33"/>
+      <c r="T17" s="33"/>
+      <c r="U17" s="33"/>
+      <c r="V17" s="33"/>
+      <c r="W17" s="33"/>
+      <c r="Y17" s="34"/>
+      <c r="Z17" s="34"/>
+      <c r="AA17" s="34"/>
+      <c r="AB17" s="34"/>
+      <c r="AC17" s="34"/>
+      <c r="AD17" s="34"/>
+      <c r="AF17" s="35"/>
+      <c r="AG17" s="35"/>
+      <c r="AH17" s="35"/>
+      <c r="AI17" s="35"/>
+      <c r="AJ17" s="35"/>
+      <c r="AK17" s="35"/>
+      <c r="AM17" s="36"/>
+      <c r="AN17" s="36"/>
+      <c r="AO17" s="36"/>
+      <c r="AP17" s="36"/>
+      <c r="AQ17" s="36"/>
+      <c r="AR17" s="36"/>
     </row>
     <row r="18" spans="3:44" ht="18" customHeight="1"/>
     <row r="19" spans="3:44" ht="4" customHeight="1"/>
     <row r="20" spans="3:44" ht="18" customHeight="1">
-      <c r="C20" s="36" t="s">
+      <c r="C20" s="37" t="s">
         <v>238</v>
       </c>
-      <c r="D20" s="36"/>
-      <c r="E20" s="36"/>
-      <c r="F20" s="36"/>
-      <c r="G20" s="36"/>
-      <c r="H20" s="36"/>
-      <c r="I20" s="36"/>
-      <c r="J20" s="36"/>
-      <c r="K20" s="36"/>
-      <c r="L20" s="36"/>
-      <c r="M20" s="36"/>
-      <c r="N20" s="36"/>
-      <c r="O20" s="36" t="s">
+      <c r="D20" s="37"/>
+      <c r="E20" s="37"/>
+      <c r="F20" s="37"/>
+      <c r="G20" s="37"/>
+      <c r="H20" s="37"/>
+      <c r="I20" s="37"/>
+      <c r="J20" s="37"/>
+      <c r="K20" s="37"/>
+      <c r="L20" s="37"/>
+      <c r="M20" s="37"/>
+      <c r="N20" s="37"/>
+      <c r="O20" s="37" t="s">
         <v>239</v>
       </c>
-      <c r="P20" s="36"/>
-      <c r="Q20" s="36"/>
-      <c r="R20" s="36"/>
-      <c r="S20" s="36"/>
-      <c r="T20" s="36"/>
-      <c r="U20" s="36"/>
-      <c r="V20" s="36"/>
-      <c r="W20" s="36"/>
-      <c r="X20" s="36"/>
-      <c r="Y20" s="36"/>
-      <c r="Z20" s="36"/>
-      <c r="AA20" s="36" t="s">
+      <c r="P20" s="37"/>
+      <c r="Q20" s="37"/>
+      <c r="R20" s="37"/>
+      <c r="S20" s="37"/>
+      <c r="T20" s="37"/>
+      <c r="U20" s="37"/>
+      <c r="V20" s="37"/>
+      <c r="W20" s="37"/>
+      <c r="X20" s="37"/>
+      <c r="Y20" s="37"/>
+      <c r="Z20" s="37"/>
+      <c r="AA20" s="37" t="s">
         <v>240</v>
       </c>
-      <c r="AB20" s="36"/>
-      <c r="AC20" s="36"/>
-      <c r="AD20" s="36"/>
-      <c r="AE20" s="36"/>
-      <c r="AF20" s="36"/>
-      <c r="AG20" s="36"/>
-      <c r="AH20" s="36"/>
-      <c r="AI20" s="36"/>
-      <c r="AJ20" s="36"/>
-      <c r="AK20" s="36"/>
-      <c r="AL20" s="36"/>
+      <c r="AB20" s="37"/>
+      <c r="AC20" s="37"/>
+      <c r="AD20" s="37"/>
+      <c r="AE20" s="37"/>
+      <c r="AF20" s="37"/>
+      <c r="AG20" s="37"/>
+      <c r="AH20" s="37"/>
+      <c r="AI20" s="37"/>
+      <c r="AJ20" s="37"/>
+      <c r="AK20" s="37"/>
+      <c r="AL20" s="37"/>
     </row>
     <row r="21" spans="3:44" ht="6" customHeight="1">
-      <c r="C21" s="36"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="36"/>
-      <c r="F21" s="36"/>
-      <c r="G21" s="36"/>
-      <c r="H21" s="36"/>
-      <c r="I21" s="36"/>
-      <c r="J21" s="36"/>
-      <c r="K21" s="36"/>
-      <c r="L21" s="36"/>
-      <c r="M21" s="36"/>
-      <c r="N21" s="36"/>
-      <c r="O21" s="36"/>
-      <c r="P21" s="36"/>
-      <c r="Q21" s="36"/>
-      <c r="R21" s="36"/>
-      <c r="S21" s="36"/>
-      <c r="T21" s="36"/>
-      <c r="U21" s="36"/>
-      <c r="V21" s="36"/>
-      <c r="W21" s="36"/>
-      <c r="X21" s="36"/>
-      <c r="Y21" s="36"/>
-      <c r="Z21" s="36"/>
-      <c r="AA21" s="36"/>
-      <c r="AB21" s="36"/>
-      <c r="AC21" s="36"/>
-      <c r="AD21" s="36"/>
-      <c r="AE21" s="36"/>
-      <c r="AF21" s="36"/>
-      <c r="AG21" s="36"/>
-      <c r="AH21" s="36"/>
-      <c r="AI21" s="36"/>
-      <c r="AJ21" s="36"/>
-      <c r="AK21" s="36"/>
-      <c r="AL21" s="36"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="37"/>
+      <c r="I21" s="37"/>
+      <c r="J21" s="37"/>
+      <c r="K21" s="37"/>
+      <c r="L21" s="37"/>
+      <c r="M21" s="37"/>
+      <c r="N21" s="37"/>
+      <c r="O21" s="37"/>
+      <c r="P21" s="37"/>
+      <c r="Q21" s="37"/>
+      <c r="R21" s="37"/>
+      <c r="S21" s="37"/>
+      <c r="T21" s="37"/>
+      <c r="U21" s="37"/>
+      <c r="V21" s="37"/>
+      <c r="W21" s="37"/>
+      <c r="X21" s="37"/>
+      <c r="Y21" s="37"/>
+      <c r="Z21" s="37"/>
+      <c r="AA21" s="37"/>
+      <c r="AB21" s="37"/>
+      <c r="AC21" s="37"/>
+      <c r="AD21" s="37"/>
+      <c r="AE21" s="37"/>
+      <c r="AF21" s="37"/>
+      <c r="AG21" s="37"/>
+      <c r="AH21" s="37"/>
+      <c r="AI21" s="37"/>
+      <c r="AJ21" s="37"/>
+      <c r="AK21" s="37"/>
+      <c r="AL21" s="37"/>
     </row>
     <row r="22" spans="3:44" ht="16" customHeight="1"/>
-    <row r="23" spans="3:44" ht="6" customHeight="1"/>
-    <row r="24" spans="3:44" ht="6" customHeight="1"/>
-    <row r="25" spans="3:44" ht="6" customHeight="1"/>
-    <row r="26" spans="3:44" ht="6" customHeight="1"/>
-    <row r="27" spans="3:44" ht="6" customHeight="1"/>
-    <row r="28" spans="3:44" ht="6" customHeight="1"/>
-    <row r="29" spans="3:44" ht="6" customHeight="1"/>
-    <row r="30" spans="3:44" ht="6" customHeight="1"/>
-    <row r="31" spans="3:44" ht="6" customHeight="1"/>
-    <row r="32" spans="3:44" ht="6" customHeight="1"/>
-    <row r="33" spans="3:38" ht="6" customHeight="1"/>
-    <row r="34" spans="3:38" ht="6" customHeight="1"/>
-    <row r="35" spans="3:38" ht="6" customHeight="1"/>
-    <row r="36" spans="3:38" ht="6" customHeight="1"/>
-    <row r="37" spans="3:38" ht="6" customHeight="1"/>
-    <row r="38" spans="3:38" ht="6" customHeight="1"/>
-    <row r="39" spans="3:38" ht="6" customHeight="1"/>
-    <row r="40" spans="3:38" ht="6" customHeight="1"/>
-    <row r="41" spans="3:38" ht="6" customHeight="1"/>
+    <row r="23" spans="3:44" ht="10" customHeight="1"/>
+    <row r="24" spans="3:44" ht="10" customHeight="1"/>
+    <row r="25" spans="3:44" ht="10" customHeight="1"/>
+    <row r="26" spans="3:44" ht="10" customHeight="1"/>
+    <row r="27" spans="3:44" ht="10" customHeight="1"/>
+    <row r="28" spans="3:44" ht="10" customHeight="1"/>
+    <row r="29" spans="3:44" ht="10" customHeight="1"/>
+    <row r="30" spans="3:44" ht="10" customHeight="1"/>
+    <row r="31" spans="3:44" ht="10" customHeight="1"/>
+    <row r="32" spans="3:44" ht="10" customHeight="1"/>
+    <row r="33" spans="3:38" ht="10" customHeight="1"/>
+    <row r="34" spans="3:38" ht="10" customHeight="1"/>
+    <row r="35" spans="3:38" ht="10" customHeight="1"/>
+    <row r="36" spans="3:38" ht="10" customHeight="1"/>
+    <row r="37" spans="3:38" ht="10" customHeight="1"/>
+    <row r="38" spans="3:38" ht="10" customHeight="1"/>
+    <row r="39" spans="3:38" ht="10" customHeight="1"/>
+    <row r="40" spans="3:38" ht="10" customHeight="1"/>
+    <row r="41" spans="3:38" ht="10" customHeight="1"/>
     <row r="42" spans="3:38" ht="4" customHeight="1"/>
     <row r="43" spans="3:38" ht="18" customHeight="1">
-      <c r="C43" s="36" t="s">
+      <c r="C43" s="37" t="s">
         <v>241</v>
       </c>
-      <c r="D43" s="36"/>
-      <c r="E43" s="36"/>
-      <c r="F43" s="36"/>
-      <c r="G43" s="36"/>
-      <c r="H43" s="36"/>
-      <c r="I43" s="36"/>
-      <c r="J43" s="36"/>
-      <c r="K43" s="36"/>
-      <c r="L43" s="36"/>
-      <c r="M43" s="36"/>
-      <c r="N43" s="36"/>
-      <c r="O43" s="36" t="s">
+      <c r="D43" s="37"/>
+      <c r="E43" s="37"/>
+      <c r="F43" s="37"/>
+      <c r="G43" s="37"/>
+      <c r="H43" s="37"/>
+      <c r="I43" s="37"/>
+      <c r="J43" s="37"/>
+      <c r="K43" s="37"/>
+      <c r="L43" s="37"/>
+      <c r="M43" s="37"/>
+      <c r="N43" s="37"/>
+      <c r="O43" s="37" t="s">
         <v>242</v>
       </c>
-      <c r="P43" s="36"/>
-      <c r="Q43" s="36"/>
-      <c r="R43" s="36"/>
-      <c r="S43" s="36"/>
-      <c r="T43" s="36"/>
-      <c r="U43" s="36"/>
-      <c r="V43" s="36"/>
-      <c r="W43" s="36"/>
-      <c r="X43" s="36"/>
-      <c r="Y43" s="36"/>
-      <c r="Z43" s="36"/>
-      <c r="AA43" s="36" t="s">
+      <c r="P43" s="37"/>
+      <c r="Q43" s="37"/>
+      <c r="R43" s="37"/>
+      <c r="S43" s="37"/>
+      <c r="T43" s="37"/>
+      <c r="U43" s="37"/>
+      <c r="V43" s="37"/>
+      <c r="W43" s="37"/>
+      <c r="X43" s="37"/>
+      <c r="Y43" s="37"/>
+      <c r="Z43" s="37"/>
+      <c r="AA43" s="37" t="s">
         <v>243</v>
       </c>
-      <c r="AB43" s="36"/>
-      <c r="AC43" s="36"/>
-      <c r="AD43" s="36"/>
-      <c r="AE43" s="36"/>
-      <c r="AF43" s="36"/>
-      <c r="AG43" s="36"/>
-      <c r="AH43" s="36"/>
-      <c r="AI43" s="36"/>
-      <c r="AJ43" s="36"/>
-      <c r="AK43" s="36"/>
-      <c r="AL43" s="36"/>
+      <c r="AB43" s="37"/>
+      <c r="AC43" s="37"/>
+      <c r="AD43" s="37"/>
+      <c r="AE43" s="37"/>
+      <c r="AF43" s="37"/>
+      <c r="AG43" s="37"/>
+      <c r="AH43" s="37"/>
+      <c r="AI43" s="37"/>
+      <c r="AJ43" s="37"/>
+      <c r="AK43" s="37"/>
+      <c r="AL43" s="37"/>
     </row>
     <row r="44" spans="3:38" ht="6" customHeight="1">
-      <c r="C44" s="36"/>
-      <c r="D44" s="36"/>
-      <c r="E44" s="36"/>
-      <c r="F44" s="36"/>
-      <c r="G44" s="36"/>
-      <c r="H44" s="36"/>
-      <c r="I44" s="36"/>
-      <c r="J44" s="36"/>
-      <c r="K44" s="36"/>
-      <c r="L44" s="36"/>
-      <c r="M44" s="36"/>
-      <c r="N44" s="36"/>
-      <c r="O44" s="36"/>
-      <c r="P44" s="36"/>
-      <c r="Q44" s="36"/>
-      <c r="R44" s="36"/>
-      <c r="S44" s="36"/>
-      <c r="T44" s="36"/>
-      <c r="U44" s="36"/>
-      <c r="V44" s="36"/>
-      <c r="W44" s="36"/>
-      <c r="X44" s="36"/>
-      <c r="Y44" s="36"/>
-      <c r="Z44" s="36"/>
-      <c r="AA44" s="36"/>
-      <c r="AB44" s="36"/>
-      <c r="AC44" s="36"/>
-      <c r="AD44" s="36"/>
-      <c r="AE44" s="36"/>
-      <c r="AF44" s="36"/>
-      <c r="AG44" s="36"/>
-      <c r="AH44" s="36"/>
-      <c r="AI44" s="36"/>
-      <c r="AJ44" s="36"/>
-      <c r="AK44" s="36"/>
-      <c r="AL44" s="36"/>
+      <c r="C44" s="37"/>
+      <c r="D44" s="37"/>
+      <c r="E44" s="37"/>
+      <c r="F44" s="37"/>
+      <c r="G44" s="37"/>
+      <c r="H44" s="37"/>
+      <c r="I44" s="37"/>
+      <c r="J44" s="37"/>
+      <c r="K44" s="37"/>
+      <c r="L44" s="37"/>
+      <c r="M44" s="37"/>
+      <c r="N44" s="37"/>
+      <c r="O44" s="37"/>
+      <c r="P44" s="37"/>
+      <c r="Q44" s="37"/>
+      <c r="R44" s="37"/>
+      <c r="S44" s="37"/>
+      <c r="T44" s="37"/>
+      <c r="U44" s="37"/>
+      <c r="V44" s="37"/>
+      <c r="W44" s="37"/>
+      <c r="X44" s="37"/>
+      <c r="Y44" s="37"/>
+      <c r="Z44" s="37"/>
+      <c r="AA44" s="37"/>
+      <c r="AB44" s="37"/>
+      <c r="AC44" s="37"/>
+      <c r="AD44" s="37"/>
+      <c r="AE44" s="37"/>
+      <c r="AF44" s="37"/>
+      <c r="AG44" s="37"/>
+      <c r="AH44" s="37"/>
+      <c r="AI44" s="37"/>
+      <c r="AJ44" s="37"/>
+      <c r="AK44" s="37"/>
+      <c r="AL44" s="37"/>
     </row>
     <row r="45" spans="3:38" ht="16" customHeight="1"/>
-    <row r="46" spans="3:38" ht="6" customHeight="1"/>
-    <row r="47" spans="3:38" ht="6" customHeight="1"/>
-    <row r="48" spans="3:38" ht="6" customHeight="1"/>
-    <row r="49" ht="6" customHeight="1"/>
-    <row r="50" ht="6" customHeight="1"/>
-    <row r="51" ht="6" customHeight="1"/>
-    <row r="52" ht="6" customHeight="1"/>
-    <row r="53" ht="6" customHeight="1"/>
-    <row r="54" ht="6" customHeight="1"/>
-    <row r="55" ht="6" customHeight="1"/>
-    <row r="56" ht="6" customHeight="1"/>
-    <row r="57" ht="6" customHeight="1"/>
-    <row r="58" ht="6" customHeight="1"/>
-    <row r="59" ht="6" customHeight="1"/>
-    <row r="60" ht="6" customHeight="1"/>
-    <row r="61" ht="6" customHeight="1"/>
-    <row r="62" ht="6" customHeight="1"/>
-    <row r="63" ht="6" customHeight="1"/>
-    <row r="64" ht="6" customHeight="1"/>
+    <row r="46" spans="3:38" ht="10" customHeight="1"/>
+    <row r="47" spans="3:38" ht="10" customHeight="1"/>
+    <row r="48" spans="3:38" ht="10" customHeight="1"/>
+    <row r="49" ht="10" customHeight="1"/>
+    <row r="50" ht="10" customHeight="1"/>
+    <row r="51" ht="10" customHeight="1"/>
+    <row r="52" ht="10" customHeight="1"/>
+    <row r="53" ht="10" customHeight="1"/>
+    <row r="54" ht="10" customHeight="1"/>
+    <row r="55" ht="10" customHeight="1"/>
+    <row r="56" ht="10" customHeight="1"/>
+    <row r="57" ht="10" customHeight="1"/>
+    <row r="58" ht="10" customHeight="1"/>
+    <row r="59" ht="10" customHeight="1"/>
+    <row r="60" ht="10" customHeight="1"/>
+    <row r="61" ht="10" customHeight="1"/>
+    <row r="62" ht="10" customHeight="1"/>
+    <row r="63" ht="10" customHeight="1"/>
+    <row r="64" ht="10" customHeight="1"/>
     <row r="65" ht="4" customHeight="1"/>
     <row r="66" ht="6" customHeight="1"/>
     <row r="67" ht="6" customHeight="1"/>
@@ -22852,307 +22831,307 @@
     <row r="90" spans="3:44" ht="14" customHeight="1"/>
     <row r="91" spans="3:44" ht="6" customHeight="1"/>
     <row r="92" spans="3:44" ht="18" customHeight="1">
-      <c r="C92" s="37" t="s">
+      <c r="C92" s="38" t="s">
         <v>245</v>
       </c>
-      <c r="D92" s="37"/>
-      <c r="E92" s="37"/>
-      <c r="F92" s="37"/>
-      <c r="G92" s="37"/>
-      <c r="H92" s="37"/>
-      <c r="I92" s="37"/>
-      <c r="J92" s="37" t="s">
+      <c r="D92" s="38"/>
+      <c r="E92" s="38"/>
+      <c r="F92" s="38"/>
+      <c r="G92" s="38"/>
+      <c r="H92" s="38"/>
+      <c r="I92" s="38"/>
+      <c r="J92" s="38" t="s">
         <v>248</v>
       </c>
-      <c r="K92" s="37"/>
-      <c r="L92" s="37"/>
-      <c r="M92" s="37"/>
-      <c r="N92" s="37"/>
-      <c r="O92" s="37"/>
-      <c r="P92" s="37"/>
-      <c r="Q92" s="37" t="s">
+      <c r="K92" s="38"/>
+      <c r="L92" s="38"/>
+      <c r="M92" s="38"/>
+      <c r="N92" s="38"/>
+      <c r="O92" s="38"/>
+      <c r="P92" s="38"/>
+      <c r="Q92" s="38" t="s">
         <v>251</v>
       </c>
-      <c r="R92" s="37"/>
-      <c r="S92" s="37"/>
-      <c r="T92" s="37"/>
-      <c r="U92" s="37"/>
-      <c r="V92" s="37"/>
-      <c r="W92" s="37"/>
-      <c r="X92" s="37" t="s">
+      <c r="R92" s="38"/>
+      <c r="S92" s="38"/>
+      <c r="T92" s="38"/>
+      <c r="U92" s="38"/>
+      <c r="V92" s="38"/>
+      <c r="W92" s="38"/>
+      <c r="X92" s="38" t="s">
         <v>254</v>
       </c>
-      <c r="Y92" s="37"/>
-      <c r="Z92" s="37"/>
-      <c r="AA92" s="37"/>
-      <c r="AB92" s="37"/>
-      <c r="AC92" s="37"/>
-      <c r="AD92" s="37"/>
-      <c r="AE92" s="37" t="s">
+      <c r="Y92" s="38"/>
+      <c r="Z92" s="38"/>
+      <c r="AA92" s="38"/>
+      <c r="AB92" s="38"/>
+      <c r="AC92" s="38"/>
+      <c r="AD92" s="38"/>
+      <c r="AE92" s="38" t="s">
         <v>257</v>
       </c>
-      <c r="AF92" s="37"/>
-      <c r="AG92" s="37"/>
-      <c r="AH92" s="37"/>
-      <c r="AI92" s="37"/>
-      <c r="AJ92" s="37"/>
-      <c r="AK92" s="37"/>
-      <c r="AL92" s="37" t="s">
+      <c r="AF92" s="38"/>
+      <c r="AG92" s="38"/>
+      <c r="AH92" s="38"/>
+      <c r="AI92" s="38"/>
+      <c r="AJ92" s="38"/>
+      <c r="AK92" s="38"/>
+      <c r="AL92" s="38" t="s">
         <v>229</v>
       </c>
-      <c r="AM92" s="37"/>
-      <c r="AN92" s="37"/>
-      <c r="AO92" s="37"/>
-      <c r="AP92" s="37"/>
-      <c r="AQ92" s="37"/>
-      <c r="AR92" s="37"/>
+      <c r="AM92" s="38"/>
+      <c r="AN92" s="38"/>
+      <c r="AO92" s="38"/>
+      <c r="AP92" s="38"/>
+      <c r="AQ92" s="38"/>
+      <c r="AR92" s="38"/>
     </row>
     <row r="93" spans="3:44" ht="18" customHeight="1">
-      <c r="C93" s="38" t="s">
+      <c r="C93" s="39" t="s">
         <v>246</v>
       </c>
-      <c r="D93" s="38"/>
-      <c r="E93" s="38"/>
-      <c r="F93" s="38"/>
-      <c r="G93" s="38"/>
-      <c r="H93" s="38"/>
-      <c r="I93" s="38"/>
-      <c r="J93" s="38" t="s">
+      <c r="D93" s="39"/>
+      <c r="E93" s="39"/>
+      <c r="F93" s="39"/>
+      <c r="G93" s="39"/>
+      <c r="H93" s="39"/>
+      <c r="I93" s="39"/>
+      <c r="J93" s="39" t="s">
         <v>249</v>
       </c>
-      <c r="K93" s="38"/>
-      <c r="L93" s="38"/>
-      <c r="M93" s="38"/>
-      <c r="N93" s="38"/>
-      <c r="O93" s="38"/>
-      <c r="P93" s="38"/>
-      <c r="Q93" s="38" t="s">
+      <c r="K93" s="39"/>
+      <c r="L93" s="39"/>
+      <c r="M93" s="39"/>
+      <c r="N93" s="39"/>
+      <c r="O93" s="39"/>
+      <c r="P93" s="39"/>
+      <c r="Q93" s="39" t="s">
         <v>252</v>
       </c>
-      <c r="R93" s="38"/>
-      <c r="S93" s="38"/>
-      <c r="T93" s="38"/>
-      <c r="U93" s="38"/>
-      <c r="V93" s="38"/>
-      <c r="W93" s="38"/>
-      <c r="X93" s="38" t="s">
+      <c r="R93" s="39"/>
+      <c r="S93" s="39"/>
+      <c r="T93" s="39"/>
+      <c r="U93" s="39"/>
+      <c r="V93" s="39"/>
+      <c r="W93" s="39"/>
+      <c r="X93" s="39" t="s">
         <v>255</v>
       </c>
-      <c r="Y93" s="38"/>
-      <c r="Z93" s="38"/>
-      <c r="AA93" s="38"/>
-      <c r="AB93" s="38"/>
-      <c r="AC93" s="38"/>
-      <c r="AD93" s="38"/>
-      <c r="AE93" s="38" t="s">
+      <c r="Y93" s="39"/>
+      <c r="Z93" s="39"/>
+      <c r="AA93" s="39"/>
+      <c r="AB93" s="39"/>
+      <c r="AC93" s="39"/>
+      <c r="AD93" s="39"/>
+      <c r="AE93" s="39" t="s">
         <v>258</v>
       </c>
-      <c r="AF93" s="38"/>
-      <c r="AG93" s="38"/>
-      <c r="AH93" s="38"/>
-      <c r="AI93" s="38"/>
-      <c r="AJ93" s="38"/>
-      <c r="AK93" s="38"/>
-      <c r="AL93" s="38" t="s">
+      <c r="AF93" s="39"/>
+      <c r="AG93" s="39"/>
+      <c r="AH93" s="39"/>
+      <c r="AI93" s="39"/>
+      <c r="AJ93" s="39"/>
+      <c r="AK93" s="39"/>
+      <c r="AL93" s="39" t="s">
         <v>260</v>
       </c>
-      <c r="AM93" s="38"/>
-      <c r="AN93" s="38"/>
-      <c r="AO93" s="38"/>
-      <c r="AP93" s="38"/>
-      <c r="AQ93" s="38"/>
-      <c r="AR93" s="38"/>
+      <c r="AM93" s="39"/>
+      <c r="AN93" s="39"/>
+      <c r="AO93" s="39"/>
+      <c r="AP93" s="39"/>
+      <c r="AQ93" s="39"/>
+      <c r="AR93" s="39"/>
     </row>
     <row r="94" spans="3:44" ht="18" customHeight="1">
-      <c r="C94" s="39" t="s">
+      <c r="C94" s="40" t="s">
         <v>247</v>
       </c>
-      <c r="D94" s="39"/>
-      <c r="E94" s="39"/>
-      <c r="F94" s="39"/>
-      <c r="G94" s="39"/>
-      <c r="H94" s="39"/>
-      <c r="I94" s="39"/>
-      <c r="J94" s="39" t="s">
+      <c r="D94" s="40"/>
+      <c r="E94" s="40"/>
+      <c r="F94" s="40"/>
+      <c r="G94" s="40"/>
+      <c r="H94" s="40"/>
+      <c r="I94" s="40"/>
+      <c r="J94" s="40" t="s">
         <v>250</v>
       </c>
-      <c r="K94" s="39"/>
-      <c r="L94" s="39"/>
-      <c r="M94" s="39"/>
-      <c r="N94" s="39"/>
-      <c r="O94" s="39"/>
-      <c r="P94" s="39"/>
-      <c r="Q94" s="39" t="s">
+      <c r="K94" s="40"/>
+      <c r="L94" s="40"/>
+      <c r="M94" s="40"/>
+      <c r="N94" s="40"/>
+      <c r="O94" s="40"/>
+      <c r="P94" s="40"/>
+      <c r="Q94" s="40" t="s">
         <v>253</v>
       </c>
-      <c r="R94" s="39"/>
-      <c r="S94" s="39"/>
-      <c r="T94" s="39"/>
-      <c r="U94" s="39"/>
-      <c r="V94" s="39"/>
-      <c r="W94" s="39"/>
-      <c r="X94" s="39" t="s">
+      <c r="R94" s="40"/>
+      <c r="S94" s="40"/>
+      <c r="T94" s="40"/>
+      <c r="U94" s="40"/>
+      <c r="V94" s="40"/>
+      <c r="W94" s="40"/>
+      <c r="X94" s="40" t="s">
         <v>256</v>
       </c>
-      <c r="Y94" s="39"/>
-      <c r="Z94" s="39"/>
-      <c r="AA94" s="39"/>
-      <c r="AB94" s="39"/>
-      <c r="AC94" s="39"/>
-      <c r="AD94" s="39"/>
-      <c r="AE94" s="39" t="s">
+      <c r="Y94" s="40"/>
+      <c r="Z94" s="40"/>
+      <c r="AA94" s="40"/>
+      <c r="AB94" s="40"/>
+      <c r="AC94" s="40"/>
+      <c r="AD94" s="40"/>
+      <c r="AE94" s="40" t="s">
         <v>259</v>
       </c>
-      <c r="AF94" s="39"/>
-      <c r="AG94" s="39"/>
-      <c r="AH94" s="39"/>
-      <c r="AI94" s="39"/>
-      <c r="AJ94" s="39"/>
-      <c r="AK94" s="39"/>
-      <c r="AL94" s="39" t="s">
+      <c r="AF94" s="40"/>
+      <c r="AG94" s="40"/>
+      <c r="AH94" s="40"/>
+      <c r="AI94" s="40"/>
+      <c r="AJ94" s="40"/>
+      <c r="AK94" s="40"/>
+      <c r="AL94" s="40" t="s">
         <v>261</v>
       </c>
-      <c r="AM94" s="39"/>
-      <c r="AN94" s="39"/>
-      <c r="AO94" s="39"/>
-      <c r="AP94" s="39"/>
-      <c r="AQ94" s="39"/>
-      <c r="AR94" s="39"/>
+      <c r="AM94" s="40"/>
+      <c r="AN94" s="40"/>
+      <c r="AO94" s="40"/>
+      <c r="AP94" s="40"/>
+      <c r="AQ94" s="40"/>
+      <c r="AR94" s="40"/>
     </row>
     <row r="95" spans="3:44" ht="18" customHeight="1">
-      <c r="C95" s="39"/>
-      <c r="D95" s="39"/>
-      <c r="E95" s="39"/>
-      <c r="F95" s="39"/>
-      <c r="G95" s="39"/>
-      <c r="H95" s="39"/>
-      <c r="I95" s="39"/>
-      <c r="J95" s="39"/>
-      <c r="K95" s="39"/>
-      <c r="L95" s="39"/>
-      <c r="M95" s="39"/>
-      <c r="N95" s="39"/>
-      <c r="O95" s="39"/>
-      <c r="P95" s="39"/>
-      <c r="Q95" s="39"/>
-      <c r="R95" s="39"/>
-      <c r="S95" s="39"/>
-      <c r="T95" s="39"/>
-      <c r="U95" s="39"/>
-      <c r="V95" s="39"/>
-      <c r="W95" s="39"/>
-      <c r="X95" s="39"/>
-      <c r="Y95" s="39"/>
-      <c r="Z95" s="39"/>
-      <c r="AA95" s="39"/>
-      <c r="AB95" s="39"/>
-      <c r="AC95" s="39"/>
-      <c r="AD95" s="39"/>
-      <c r="AE95" s="39"/>
-      <c r="AF95" s="39"/>
-      <c r="AG95" s="39"/>
-      <c r="AH95" s="39"/>
-      <c r="AI95" s="39"/>
-      <c r="AJ95" s="39"/>
-      <c r="AK95" s="39"/>
-      <c r="AL95" s="39"/>
-      <c r="AM95" s="39"/>
-      <c r="AN95" s="39"/>
-      <c r="AO95" s="39"/>
-      <c r="AP95" s="39"/>
-      <c r="AQ95" s="39"/>
-      <c r="AR95" s="39"/>
+      <c r="C95" s="40"/>
+      <c r="D95" s="40"/>
+      <c r="E95" s="40"/>
+      <c r="F95" s="40"/>
+      <c r="G95" s="40"/>
+      <c r="H95" s="40"/>
+      <c r="I95" s="40"/>
+      <c r="J95" s="40"/>
+      <c r="K95" s="40"/>
+      <c r="L95" s="40"/>
+      <c r="M95" s="40"/>
+      <c r="N95" s="40"/>
+      <c r="O95" s="40"/>
+      <c r="P95" s="40"/>
+      <c r="Q95" s="40"/>
+      <c r="R95" s="40"/>
+      <c r="S95" s="40"/>
+      <c r="T95" s="40"/>
+      <c r="U95" s="40"/>
+      <c r="V95" s="40"/>
+      <c r="W95" s="40"/>
+      <c r="X95" s="40"/>
+      <c r="Y95" s="40"/>
+      <c r="Z95" s="40"/>
+      <c r="AA95" s="40"/>
+      <c r="AB95" s="40"/>
+      <c r="AC95" s="40"/>
+      <c r="AD95" s="40"/>
+      <c r="AE95" s="40"/>
+      <c r="AF95" s="40"/>
+      <c r="AG95" s="40"/>
+      <c r="AH95" s="40"/>
+      <c r="AI95" s="40"/>
+      <c r="AJ95" s="40"/>
+      <c r="AK95" s="40"/>
+      <c r="AL95" s="40"/>
+      <c r="AM95" s="40"/>
+      <c r="AN95" s="40"/>
+      <c r="AO95" s="40"/>
+      <c r="AP95" s="40"/>
+      <c r="AQ95" s="40"/>
+      <c r="AR95" s="40"/>
     </row>
     <row r="96" spans="3:44" ht="6" customHeight="1"/>
     <row r="97" spans="3:44" ht="22" customHeight="1">
-      <c r="C97" s="40" t="s">
+      <c r="C97" s="41" t="s">
         <v>262</v>
       </c>
-      <c r="D97" s="40"/>
-      <c r="E97" s="40"/>
-      <c r="F97" s="40"/>
-      <c r="G97" s="40"/>
-      <c r="H97" s="40"/>
-      <c r="I97" s="40"/>
-      <c r="J97" s="40"/>
-      <c r="K97" s="40"/>
-      <c r="L97" s="40"/>
-      <c r="M97" s="40"/>
-      <c r="N97" s="40"/>
-      <c r="O97" s="40"/>
-      <c r="P97" s="40"/>
-      <c r="Q97" s="40"/>
-      <c r="R97" s="40"/>
-      <c r="S97" s="40"/>
-      <c r="T97" s="40"/>
-      <c r="U97" s="40"/>
-      <c r="V97" s="40"/>
-      <c r="W97" s="40"/>
-      <c r="X97" s="40"/>
-      <c r="Y97" s="40"/>
-      <c r="Z97" s="40"/>
-      <c r="AA97" s="40"/>
-      <c r="AB97" s="40"/>
-      <c r="AC97" s="40"/>
-      <c r="AD97" s="40"/>
-      <c r="AE97" s="40"/>
-      <c r="AF97" s="40"/>
-      <c r="AG97" s="40"/>
-      <c r="AH97" s="40"/>
-      <c r="AI97" s="40"/>
-      <c r="AJ97" s="40"/>
-      <c r="AK97" s="40"/>
-      <c r="AL97" s="40"/>
-      <c r="AM97" s="40"/>
-      <c r="AN97" s="40"/>
-      <c r="AO97" s="40"/>
-      <c r="AP97" s="40"/>
-      <c r="AQ97" s="40"/>
-      <c r="AR97" s="40"/>
+      <c r="D97" s="41"/>
+      <c r="E97" s="41"/>
+      <c r="F97" s="41"/>
+      <c r="G97" s="41"/>
+      <c r="H97" s="41"/>
+      <c r="I97" s="41"/>
+      <c r="J97" s="41"/>
+      <c r="K97" s="41"/>
+      <c r="L97" s="41"/>
+      <c r="M97" s="41"/>
+      <c r="N97" s="41"/>
+      <c r="O97" s="41"/>
+      <c r="P97" s="41"/>
+      <c r="Q97" s="41"/>
+      <c r="R97" s="41"/>
+      <c r="S97" s="41"/>
+      <c r="T97" s="41"/>
+      <c r="U97" s="41"/>
+      <c r="V97" s="41"/>
+      <c r="W97" s="41"/>
+      <c r="X97" s="41"/>
+      <c r="Y97" s="41"/>
+      <c r="Z97" s="41"/>
+      <c r="AA97" s="41"/>
+      <c r="AB97" s="41"/>
+      <c r="AC97" s="41"/>
+      <c r="AD97" s="41"/>
+      <c r="AE97" s="41"/>
+      <c r="AF97" s="41"/>
+      <c r="AG97" s="41"/>
+      <c r="AH97" s="41"/>
+      <c r="AI97" s="41"/>
+      <c r="AJ97" s="41"/>
+      <c r="AK97" s="41"/>
+      <c r="AL97" s="41"/>
+      <c r="AM97" s="41"/>
+      <c r="AN97" s="41"/>
+      <c r="AO97" s="41"/>
+      <c r="AP97" s="41"/>
+      <c r="AQ97" s="41"/>
+      <c r="AR97" s="41"/>
     </row>
     <row r="98" spans="3:44" ht="22" customHeight="1">
-      <c r="C98" s="40"/>
-      <c r="D98" s="40"/>
-      <c r="E98" s="40"/>
-      <c r="F98" s="40"/>
-      <c r="G98" s="40"/>
-      <c r="H98" s="40"/>
-      <c r="I98" s="40"/>
-      <c r="J98" s="40"/>
-      <c r="K98" s="40"/>
-      <c r="L98" s="40"/>
-      <c r="M98" s="40"/>
-      <c r="N98" s="40"/>
-      <c r="O98" s="40"/>
-      <c r="P98" s="40"/>
-      <c r="Q98" s="40"/>
-      <c r="R98" s="40"/>
-      <c r="S98" s="40"/>
-      <c r="T98" s="40"/>
-      <c r="U98" s="40"/>
-      <c r="V98" s="40"/>
-      <c r="W98" s="40"/>
-      <c r="X98" s="40"/>
-      <c r="Y98" s="40"/>
-      <c r="Z98" s="40"/>
-      <c r="AA98" s="40"/>
-      <c r="AB98" s="40"/>
-      <c r="AC98" s="40"/>
-      <c r="AD98" s="40"/>
-      <c r="AE98" s="40"/>
-      <c r="AF98" s="40"/>
-      <c r="AG98" s="40"/>
-      <c r="AH98" s="40"/>
-      <c r="AI98" s="40"/>
-      <c r="AJ98" s="40"/>
-      <c r="AK98" s="40"/>
-      <c r="AL98" s="40"/>
-      <c r="AM98" s="40"/>
-      <c r="AN98" s="40"/>
-      <c r="AO98" s="40"/>
-      <c r="AP98" s="40"/>
-      <c r="AQ98" s="40"/>
-      <c r="AR98" s="40"/>
+      <c r="C98" s="41"/>
+      <c r="D98" s="41"/>
+      <c r="E98" s="41"/>
+      <c r="F98" s="41"/>
+      <c r="G98" s="41"/>
+      <c r="H98" s="41"/>
+      <c r="I98" s="41"/>
+      <c r="J98" s="41"/>
+      <c r="K98" s="41"/>
+      <c r="L98" s="41"/>
+      <c r="M98" s="41"/>
+      <c r="N98" s="41"/>
+      <c r="O98" s="41"/>
+      <c r="P98" s="41"/>
+      <c r="Q98" s="41"/>
+      <c r="R98" s="41"/>
+      <c r="S98" s="41"/>
+      <c r="T98" s="41"/>
+      <c r="U98" s="41"/>
+      <c r="V98" s="41"/>
+      <c r="W98" s="41"/>
+      <c r="X98" s="41"/>
+      <c r="Y98" s="41"/>
+      <c r="Z98" s="41"/>
+      <c r="AA98" s="41"/>
+      <c r="AB98" s="41"/>
+      <c r="AC98" s="41"/>
+      <c r="AD98" s="41"/>
+      <c r="AE98" s="41"/>
+      <c r="AF98" s="41"/>
+      <c r="AG98" s="41"/>
+      <c r="AH98" s="41"/>
+      <c r="AI98" s="41"/>
+      <c r="AJ98" s="41"/>
+      <c r="AK98" s="41"/>
+      <c r="AL98" s="41"/>
+      <c r="AM98" s="41"/>
+      <c r="AN98" s="41"/>
+      <c r="AO98" s="41"/>
+      <c r="AP98" s="41"/>
+      <c r="AQ98" s="41"/>
+      <c r="AR98" s="41"/>
     </row>
     <row r="99" spans="3:44" ht="6" customHeight="1"/>
     <row r="100" spans="3:44" ht="6" customHeight="1"/>
@@ -23654,6 +23633,7 @@
     <row r="264" spans="1:2" hidden="1"/>
     <row r="265" spans="1:2" hidden="1"/>
   </sheetData>
+  <sheetProtection sheet="1" scenarios="1"/>
   <mergeCells count="61">
     <mergeCell ref="C1:V4"/>
     <mergeCell ref="W1:AM4"/>
@@ -23790,96 +23770,96 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="20" customHeight="1">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="41" t="s">
         <v>263</v>
       </c>
-      <c r="B1" s="40"/>
+      <c r="B1" s="41"/>
     </row>
     <row r="2" spans="1:2" ht="20" customHeight="1">
-      <c r="A2" s="40"/>
-      <c r="B2" s="40"/>
+      <c r="A2" s="41"/>
+      <c r="B2" s="41"/>
     </row>
     <row r="3" spans="1:2" ht="20" customHeight="1">
-      <c r="A3" s="40"/>
-      <c r="B3" s="40"/>
+      <c r="A3" s="41"/>
+      <c r="B3" s="41"/>
     </row>
     <row r="5" spans="1:2" ht="50" customHeight="1">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="42" t="s">
         <v>264</v>
       </c>
-      <c r="B5" s="42" t="s">
+      <c r="B5" s="43" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="50" customHeight="1">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="44" t="s">
         <v>266</v>
       </c>
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="45" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="50" customHeight="1">
-      <c r="A7" s="41" t="s">
+      <c r="A7" s="42" t="s">
         <v>268</v>
       </c>
-      <c r="B7" s="42" t="s">
+      <c r="B7" s="43" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="50" customHeight="1">
-      <c r="A8" s="43" t="s">
+      <c r="A8" s="44" t="s">
         <v>270</v>
       </c>
-      <c r="B8" s="44" t="s">
+      <c r="B8" s="45" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="50" customHeight="1">
-      <c r="A9" s="41" t="s">
+      <c r="A9" s="42" t="s">
         <v>272</v>
       </c>
-      <c r="B9" s="42" t="s">
+      <c r="B9" s="43" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="50" customHeight="1">
-      <c r="A10" s="43" t="s">
+      <c r="A10" s="44" t="s">
         <v>274</v>
       </c>
-      <c r="B10" s="44" t="s">
+      <c r="B10" s="45" t="s">
         <v>275</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="50" customHeight="1">
-      <c r="A11" s="41" t="s">
+      <c r="A11" s="42" t="s">
         <v>276</v>
       </c>
-      <c r="B11" s="42" t="s">
+      <c r="B11" s="43" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="50" customHeight="1">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="44" t="s">
         <v>278</v>
       </c>
-      <c r="B12" s="44" t="s">
+      <c r="B12" s="45" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="50" customHeight="1">
-      <c r="A13" s="41" t="s">
+      <c r="A13" s="42" t="s">
         <v>280</v>
       </c>
-      <c r="B13" s="42" t="s">
+      <c r="B13" s="43" t="s">
         <v>281</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="50" customHeight="1">
-      <c r="A14" s="43" t="s">
+      <c r="A14" s="44" t="s">
         <v>282</v>
       </c>
-      <c r="B14" s="44" t="s">
+      <c r="B14" s="45" t="s">
         <v>283</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: HSE dashboard charts now render + cleaner layout
- Charts were blank because their source data sat in hidden rows and
  xlsxwriter skips hidden cells when plotting. Added show_hidden_data()
  to all six charts so they plot correctly.
- Resized charts (348x252) and switched to fixed positioning so they sit
  inside their panels instead of overflowing into neighbouring sections.

https://claude.ai/code/session_01GWgEEwfYnssivXBBGdjyqm
</commit_message>
<xml_diff>
--- a/static/resources/HSE-Complete-Dashboard.xlsx
+++ b/static/resources/HSE-Complete-Dashboard.xlsx
@@ -1798,7 +1798,6 @@
         </a:p>
       </c:txPr>
     </c:legend>
-    <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1996,7 +1995,6 @@
         </a:ln>
       </c:spPr>
     </c:plotArea>
-    <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2194,7 +2192,6 @@
         </a:ln>
       </c:spPr>
     </c:plotArea>
-    <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2416,7 +2413,6 @@
         </a:ln>
       </c:spPr>
     </c:plotArea>
-    <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2584,7 +2580,6 @@
         </a:ln>
       </c:spPr>
     </c:plotArea>
-    <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2764,7 +2759,6 @@
         </a:ln>
       </c:spPr>
     </c:plotArea>
-    <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2784,18 +2778,18 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>57150</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2814,18 +2808,18 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>57150</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2844,18 +2838,18 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>26</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>57150</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>40</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2874,18 +2868,18 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>57150</xdr:colOff>
       <xdr:row>44</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2904,18 +2898,18 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>57150</xdr:colOff>
       <xdr:row>44</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2934,18 +2928,18 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>26</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>57150</xdr:colOff>
       <xdr:row>44</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>40</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>